<commit_message>
Przegląd bezpieczeństwa: funkcje z sekretami tylko dla serwera, limity prób w bazie, CSP, retencja danych; strony prawne; dokumenty RODO; poradnik zaktualizowany
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CLtcebTdiTD95Zxw3a2jtX
</commit_message>
<xml_diff>
--- a/docs/poradnik/Ostoja-scenariusze-testow.xlsx
+++ b/docs/poradnik/Ostoja-scenariusze-testow.xlsx
@@ -19,7 +19,7 @@
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">Błędy!$A$1:$M$200</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Titles" vbProcedure="false">Podsumowanie!$1:$1</definedName>
     <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Titles" vbProcedure="false">Scenariusze!$1:$1</definedName>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Scenariusze!$A$1:$K$32</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Scenariusze!$A$1:$K$40</definedName>
     <definedName function="false" hidden="false" localSheetId="4" name="_xlnm.Print_Titles" vbProcedure="false">Spotkania!$1:$1</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -32,12 +32,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="252">
   <si>
     <t xml:space="preserve">Ostoja – testy wersji testowej</t>
   </si>
   <si>
-    <t xml:space="preserve">Arkusz do poradnika „Ostoja-poradnik-wersji-testowej.docx”. Stan na 15 października 2026. Tylko dane fikcyjne.</t>
+    <t xml:space="preserve">Arkusz do poradnika „Ostoja-poradnik-wersji-testowej.docx”. Stan na 16 października 2026. Tylko dane fikcyjne.</t>
   </si>
   <si>
     <t xml:space="preserve">Zakładka</t>
@@ -49,7 +49,7 @@
     <t xml:space="preserve">Scenariusze</t>
   </si>
   <si>
-    <t xml:space="preserve">31 scenariuszy z poradnika (rozdział 5). Przy każdym wybierz Wynik z listy (OK, Błąd, Nie sprawdzono), wpisz datę, tester i numer błędu. Wypełniasz tylko żółte kolumny.</t>
+    <t xml:space="preserve">39 scenariuszy z poradnika (rozdział 5). Przy każdym wybierz Wynik z listy (OK, Błąd, Nie sprawdzono), wpisz datę, tester i numer błędu. Wypełniasz tylko żółte kolumny.</t>
   </si>
   <si>
     <t xml:space="preserve">Podsumowanie</t>
@@ -172,10 +172,10 @@
     <t xml:space="preserve">Prośba o kontakt do wybranego zakładu</t>
   </si>
   <si>
-    <t xml:space="preserve">Wybierz ten zakład (Cisza) → wpisz fikcyjne dane, np. Jan Testowy, 600 100 200 → zaznacz zgodę → Poproś o kontakt.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ekran „Zapytanie wysłane” z nazwą zakładu i informacją o 15 minutach.</t>
+    <t xml:space="preserve">Wybierz ten zakład (Cisza) → wpisz fikcyjne dane, np. Jan Testowy, 600 100 200 → zaznacz zgodę → Poproś o kontakt → wpisz kod z SMS-a (w wersji testowej kod jest na ekranie) → Potwierdź i wyślij zapytanie.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ekran „Wpisz kod z SMS-a” z zamaskowanym numerem, potem „Zapytanie wysłane” z nazwą zakładu i informacją o 15 minutach.</t>
   </si>
   <si>
     <t xml:space="preserve">R5</t>
@@ -184,7 +184,7 @@
     <t xml:space="preserve">Zapytanie do 3 najbliższych</t>
   </si>
   <si>
-    <t xml:space="preserve">Powtórz R1 i na dole listy kliknij Wyślij do 3 najbliższych → wyślij formularz.</t>
+    <t xml:space="preserve">Powtórz R1 i na dole listy kliknij Wyślij do 3 najbliższych → wyślij formularz → wpisz kod.</t>
   </si>
   <si>
     <t xml:space="preserve">Potwierdzenie bez nazwy zakładu. Zapytanie widzą trzy najbliższe zakłady.</t>
@@ -256,6 +256,18 @@
     <t xml:space="preserve">Pasek „Brak połączenia z internetem…”.</t>
   </si>
   <si>
+    <t xml:space="preserve">R11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zły kod SMS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W kroku z kodem wpisz 000000 (albo inny zły kod).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">„Nieprawidłowy kod…”; po 5 złych próbach „Za dużo prób” i powrót do formularza. Zapytanie nie trafia do zakładów.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Z1</t>
   </si>
   <si>
@@ -428,6 +440,102 @@
   </si>
   <si>
     <t xml:space="preserve">250 zł netto za każde zlecenie z Ostoi z podpisaną umową; zlecenia spoza Ostoi bez opłaty.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Z14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zaproszenie pracownika</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anna, potem nowa osoba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zespół → wpisz imię, e-mail (np. nowy@cisza.test), rolę Biuro → Utwórz zaproszenie → skopiuj link → otwórz go w oknie prywatnym → Przyjmij zaproszenie.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Link zaproszenia z przyciskami Kopiuj/SMS/E-mail; po przyjęciu w wersji testowej z Supabase – link logowania na e-mail, bez Supabase – od razu panel. Nowa osoba na liście zespołu.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Z15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Odebranie dostępu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zespół → przy nowej osobie Odbierz dostęp → Potwierdzam → Odbierz dostęp.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">„Dostęp odebrany.”; przy następnym kliknięciu ta osoba trafia na stronę logowania.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Administracja</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dodanie partnera</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ola Maj</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zaloguj się → Dodaj partnera → nazwa, NIP (10 cyfr), miasto, adres, telefon, e-mail → Dodaj zakład.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Karta zakładu ze statusem „Do weryfikacji”; zakład nie pojawia się rodzinom. Ten sam NIP drugi raz – odmowa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zaproszenie właściciela</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Karta zakładu → Zaproś do panelu (rola Właściciel) → wyślij link → właściciel przyjmuje i loguje się.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Właściciel w „Osoby w panelu”; po zalogowaniu widzi swój zakład, uzupełnia cennik.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weryfikacja i wstrzymanie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Karta zakładu → zaznacz „Sprawdziłem dokumenty” → Zweryfikuj zakład; potem Wstrzymaj zakład.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Po weryfikacji (i z pełnym cennikiem) zakład jest na liście ofert; po wstrzymaniu znika i nie dostaje zapytań.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zapytania do opiekuna</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Do opiekuna → zadzwoń (fikcyjny numer) → notatka → Oznacz jako obsłużone.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zapytanie Renaty Testowej z telefonem; po oznaczeniu przechodzi do „Obsłużone w ostatnim tygodniu”.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rozliczenia i dostęp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ola Maj, potem Anna</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rozliczenia (bieżący miesiąc) → potem zaloguj się jako Anna i otwórz /admin.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lista zakładów z liczbą zleceń i kwotą do faktury; Anna nie wchodzi do administracji.</t>
   </si>
   <si>
     <t xml:space="preserve">L1</t>
@@ -1317,7 +1425,7 @@
     <tabColor rgb="FF3F5650"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:K32"/>
+  <dimension ref="A1:K40"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -1449,7 +1557,7 @@
       <c r="J4" s="5"/>
       <c r="K4" s="5"/>
     </row>
-    <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
         <v>44</v>
       </c>
@@ -1638,24 +1746,24 @@
       <c r="J11" s="5"/>
       <c r="K11" s="5"/>
     </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
         <v>74</v>
       </c>
       <c r="B12" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="D12" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E12" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="F12" s="4" t="s">
         <v>77</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>79</v>
       </c>
       <c r="G12" s="4" t="s">
         <v>35</v>
@@ -1667,16 +1775,16 @@
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C13" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="B13" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="C13" s="7" t="s">
+      <c r="D13" s="4" t="s">
         <v>81</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>77</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>82</v>
@@ -1697,67 +1805,67 @@
         <v>84</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C14" s="7" t="s">
         <v>85</v>
       </c>
       <c r="D14" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E14" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="F14" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="F14" s="4" t="s">
-        <v>88</v>
-      </c>
       <c r="G14" s="4" t="s">
-        <v>89</v>
+        <v>35</v>
       </c>
       <c r="H14" s="5"/>
       <c r="I14" s="8"/>
       <c r="J14" s="5"/>
       <c r="K14" s="5"/>
     </row>
-    <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="D15" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="B15" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="C15" s="7" t="s">
+      <c r="E15" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="D15" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="E15" s="4" t="s">
+      <c r="F15" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="F15" s="4" t="s">
+      <c r="G15" s="4" t="s">
         <v>93</v>
-      </c>
-      <c r="G15" s="4" t="s">
-        <v>89</v>
       </c>
       <c r="H15" s="5"/>
       <c r="I15" s="8"/>
       <c r="J15" s="5"/>
       <c r="K15" s="5"/>
     </row>
-    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
         <v>94</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C16" s="7" t="s">
         <v>95</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="E16" s="4" t="s">
         <v>96</v>
@@ -1766,7 +1874,7 @@
         <v>97</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="H16" s="5"/>
       <c r="I16" s="8"/>
@@ -1778,13 +1886,13 @@
         <v>98</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C17" s="7" t="s">
         <v>99</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>100</v>
@@ -1793,7 +1901,7 @@
         <v>101</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="H17" s="5"/>
       <c r="I17" s="8"/>
@@ -1805,13 +1913,13 @@
         <v>102</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C18" s="7" t="s">
         <v>103</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>104</v>
@@ -1820,25 +1928,25 @@
         <v>105</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>35</v>
+        <v>93</v>
       </c>
       <c r="H18" s="5"/>
       <c r="I18" s="8"/>
       <c r="J18" s="5"/>
       <c r="K18" s="5"/>
     </row>
-    <row r="19" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
         <v>106</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C19" s="7" t="s">
         <v>107</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="E19" s="4" t="s">
         <v>108</v>
@@ -1847,25 +1955,25 @@
         <v>109</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>89</v>
+        <v>35</v>
       </c>
       <c r="H19" s="5"/>
       <c r="I19" s="8"/>
       <c r="J19" s="5"/>
       <c r="K19" s="5"/>
     </row>
-    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
         <v>110</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C20" s="7" t="s">
         <v>111</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>112</v>
@@ -1874,7 +1982,7 @@
         <v>113</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="H20" s="5"/>
       <c r="I20" s="8"/>
@@ -1886,13 +1994,13 @@
         <v>114</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C21" s="7" t="s">
         <v>115</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="E21" s="4" t="s">
         <v>116</v>
@@ -1901,7 +2009,7 @@
         <v>117</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>35</v>
+        <v>93</v>
       </c>
       <c r="H21" s="5"/>
       <c r="I21" s="8"/>
@@ -1913,19 +2021,19 @@
         <v>118</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C22" s="7" t="s">
         <v>119</v>
       </c>
       <c r="D22" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E22" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="E22" s="4" t="s">
+      <c r="F22" s="4" t="s">
         <v>121</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>122</v>
       </c>
       <c r="G22" s="4" t="s">
         <v>35</v>
@@ -1937,25 +2045,25 @@
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C23" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="B23" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="C23" s="7" t="s">
+      <c r="D23" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="E23" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="E23" s="4" t="s">
+      <c r="F23" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="F23" s="4" t="s">
-        <v>127</v>
-      </c>
       <c r="G23" s="4" t="s">
-        <v>89</v>
+        <v>35</v>
       </c>
       <c r="H23" s="5"/>
       <c r="I23" s="8"/>
@@ -1964,16 +2072,16 @@
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C24" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="B24" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="C24" s="7" t="s">
+      <c r="D24" s="4" t="s">
         <v>129</v>
-      </c>
-      <c r="D24" s="4" t="s">
-        <v>77</v>
       </c>
       <c r="E24" s="4" t="s">
         <v>130</v>
@@ -1982,7 +2090,7 @@
         <v>131</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="H24" s="5"/>
       <c r="I24" s="8"/>
@@ -1994,103 +2102,103 @@
         <v>132</v>
       </c>
       <c r="B25" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C25" s="7" t="s">
         <v>133</v>
       </c>
-      <c r="C25" s="7" t="s">
+      <c r="D25" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E25" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="D25" s="4" t="s">
+      <c r="F25" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="E25" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="F25" s="4" t="s">
-        <v>137</v>
-      </c>
       <c r="G25" s="4" t="s">
-        <v>35</v>
+        <v>93</v>
       </c>
       <c r="H25" s="5"/>
       <c r="I25" s="8"/>
       <c r="J25" s="5"/>
       <c r="K25" s="5"/>
     </row>
-    <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C26" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="D26" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="B26" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="C26" s="7" t="s">
+      <c r="E26" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="F26" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="E26" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="F26" s="4" t="s">
-        <v>142</v>
-      </c>
       <c r="G26" s="4" t="s">
-        <v>35</v>
+        <v>93</v>
       </c>
       <c r="H26" s="5"/>
       <c r="I26" s="8"/>
       <c r="J26" s="5"/>
       <c r="K26" s="5"/>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E27" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="B27" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="C27" s="7" t="s">
+      <c r="F27" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="D27" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="E27" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="F27" s="4" t="s">
-        <v>147</v>
-      </c>
       <c r="G27" s="4" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="H27" s="5"/>
       <c r="I27" s="8"/>
       <c r="J27" s="5"/>
       <c r="K27" s="5"/>
     </row>
-    <row r="28" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="D28" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="B28" s="4" t="s">
+      <c r="E28" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="C28" s="7" t="s">
+      <c r="F28" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="D28" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="E28" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="F28" s="4" t="s">
-        <v>152</v>
-      </c>
       <c r="G28" s="4" t="s">
-        <v>35</v>
+        <v>93</v>
       </c>
       <c r="H28" s="5"/>
       <c r="I28" s="8"/>
@@ -2099,25 +2207,25 @@
     </row>
     <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="E29" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="B29" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="C29" s="7" t="s">
+      <c r="F29" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="D29" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="E29" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="F29" s="4" t="s">
-        <v>156</v>
-      </c>
       <c r="G29" s="4" t="s">
-        <v>157</v>
+        <v>93</v>
       </c>
       <c r="H29" s="5"/>
       <c r="I29" s="8"/>
@@ -2126,49 +2234,49 @@
     </row>
     <row r="30" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="F30" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="B30" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="C30" s="7" t="s">
-        <v>159</v>
-      </c>
-      <c r="D30" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="E30" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="F30" s="4" t="s">
-        <v>161</v>
-      </c>
       <c r="G30" s="4" t="s">
-        <v>35</v>
+        <v>93</v>
       </c>
       <c r="H30" s="5"/>
       <c r="I30" s="8"/>
       <c r="J30" s="5"/>
       <c r="K30" s="5"/>
     </row>
-    <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="C31" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="F31" s="4" t="s">
         <v>162</v>
-      </c>
-      <c r="B31" s="4" t="s">
-        <v>163</v>
-      </c>
-      <c r="C31" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="D31" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="E31" s="4" t="s">
-        <v>165</v>
-      </c>
-      <c r="F31" s="4" t="s">
-        <v>166</v>
       </c>
       <c r="G31" s="4" t="s">
         <v>35</v>
@@ -2178,36 +2286,252 @@
       <c r="J31" s="5"/>
       <c r="K31" s="5"/>
     </row>
-    <row r="32" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="C32" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="F32" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="B32" s="4" t="s">
-        <v>163</v>
-      </c>
-      <c r="C32" s="7" t="s">
-        <v>168</v>
-      </c>
-      <c r="D32" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="E32" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="F32" s="4" t="s">
-        <v>170</v>
-      </c>
       <c r="G32" s="4" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="H32" s="5"/>
       <c r="I32" s="8"/>
       <c r="J32" s="5"/>
       <c r="K32" s="5"/>
     </row>
+    <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="C33" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="G33" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H33" s="5"/>
+      <c r="I33" s="8"/>
+      <c r="J33" s="5"/>
+      <c r="K33" s="5"/>
+    </row>
+    <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="C34" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="G34" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H34" s="5"/>
+      <c r="I34" s="8"/>
+      <c r="J34" s="5"/>
+      <c r="K34" s="5"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="C35" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="G35" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="H35" s="5"/>
+      <c r="I35" s="8"/>
+      <c r="J35" s="5"/>
+      <c r="K35" s="5"/>
+    </row>
+    <row r="36" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="C36" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="F36" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="G36" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H36" s="5"/>
+      <c r="I36" s="8"/>
+      <c r="J36" s="5"/>
+      <c r="K36" s="5"/>
+    </row>
+    <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="D37" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E37" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="F37" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="G37" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="H37" s="5"/>
+      <c r="I37" s="8"/>
+      <c r="J37" s="5"/>
+      <c r="K37" s="5"/>
+    </row>
+    <row r="38" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="C38" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E38" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="F38" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="G38" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H38" s="5"/>
+      <c r="I38" s="8"/>
+      <c r="J38" s="5"/>
+      <c r="K38" s="5"/>
+    </row>
+    <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="C39" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="G39" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H39" s="5"/>
+      <c r="I39" s="8"/>
+      <c r="J39" s="5"/>
+      <c r="K39" s="5"/>
+    </row>
+    <row r="40" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="C40" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="F40" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="G40" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="H40" s="5"/>
+      <c r="I40" s="8"/>
+      <c r="J40" s="5"/>
+      <c r="K40" s="5"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K32"/>
-  <conditionalFormatting sqref="H2:H32">
+  <autoFilter ref="A1:K40"/>
+  <conditionalFormatting sqref="H2:H40">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
       <formula>$H2="OK"</formula>
     </cfRule>
@@ -2216,11 +2540,11 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" error="Wybierz OK, Błąd albo Nie sprawdzono." errorStyle="stop" errorTitle="Wynik" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H2:H32" type="list">
+    <dataValidation allowBlank="true" error="Wybierz OK, Błąd albo Nie sprawdzono." errorStyle="stop" errorTitle="Wynik" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H2:H40" type="list">
       <formula1>"OK,Błąd,Nie sprawdzono"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Wpisz datę, np. 16.10.2026." errorStyle="stop" operator="greaterThan" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I2:I32" type="date">
+    <dataValidation allowBlank="true" error="Wpisz datę, np. 16.10.2026." errorStyle="stop" operator="greaterThan" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I2:I40" type="date">
       <formula1>DATE(2026,1,1)</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2242,7 +2566,7 @@
     <tabColor rgb="FFD8DAD7"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18"/>
@@ -2260,16 +2584,16 @@
         <v>4</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>171</v>
+        <v>207</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>172</v>
+        <v>208</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>173</v>
+        <v>209</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>174</v>
+        <v>210</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2277,20 +2601,20 @@
         <v>30</v>
       </c>
       <c r="B2" s="4" t="n">
-        <f aca="false">COUNTIF(Scenariusze!$B$2:$B$32,A2)</f>
-        <v>10</v>
+        <f aca="false">COUNTIF(Scenariusze!$B$2:$B$40,A2)</f>
+        <v>11</v>
       </c>
       <c r="C2" s="4" t="n">
-        <f aca="false">COUNTIFS(Scenariusze!$B$2:$B$32,A2,Scenariusze!$H$2:$H$32,"OK")</f>
+        <f aca="false">COUNTIFS(Scenariusze!$B$2:$B$40,A2,Scenariusze!$H$2:$H$40,"OK")</f>
         <v>0</v>
       </c>
       <c r="D2" s="4" t="n">
-        <f aca="false">COUNTIFS(Scenariusze!$B$2:$B$32,A2,Scenariusze!$H$2:$H$32,"Błąd")</f>
+        <f aca="false">COUNTIFS(Scenariusze!$B$2:$B$40,A2,Scenariusze!$H$2:$H$40,"Błąd")</f>
         <v>0</v>
       </c>
       <c r="E2" s="4" t="n">
         <f aca="false">B2-C2-D2</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F2" s="9" t="n">
         <f aca="false">IF(B2=0,0,(C2+D2)/B2)</f>
@@ -2299,23 +2623,23 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="B3" s="4" t="n">
-        <f aca="false">COUNTIF(Scenariusze!$B$2:$B$32,A3)</f>
-        <v>13</v>
+        <f aca="false">COUNTIF(Scenariusze!$B$2:$B$40,A3)</f>
+        <v>15</v>
       </c>
       <c r="C3" s="4" t="n">
-        <f aca="false">COUNTIFS(Scenariusze!$B$2:$B$32,A3,Scenariusze!$H$2:$H$32,"OK")</f>
+        <f aca="false">COUNTIFS(Scenariusze!$B$2:$B$40,A3,Scenariusze!$H$2:$H$40,"OK")</f>
         <v>0</v>
       </c>
       <c r="D3" s="4" t="n">
-        <f aca="false">COUNTIFS(Scenariusze!$B$2:$B$32,A3,Scenariusze!$H$2:$H$32,"Błąd")</f>
+        <f aca="false">COUNTIFS(Scenariusze!$B$2:$B$40,A3,Scenariusze!$H$2:$H$40,"Błąd")</f>
         <v>0</v>
       </c>
       <c r="E3" s="4" t="n">
         <f aca="false">B3-C3-D3</f>
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F3" s="9" t="n">
         <f aca="false">IF(B3=0,0,(C3+D3)/B3)</f>
@@ -2324,23 +2648,23 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>133</v>
+        <v>146</v>
       </c>
       <c r="B4" s="4" t="n">
-        <f aca="false">COUNTIF(Scenariusze!$B$2:$B$32,A4)</f>
-        <v>3</v>
+        <f aca="false">COUNTIF(Scenariusze!$B$2:$B$40,A4)</f>
+        <v>5</v>
       </c>
       <c r="C4" s="4" t="n">
-        <f aca="false">COUNTIFS(Scenariusze!$B$2:$B$32,A4,Scenariusze!$H$2:$H$32,"OK")</f>
+        <f aca="false">COUNTIFS(Scenariusze!$B$2:$B$40,A4,Scenariusze!$H$2:$H$40,"OK")</f>
         <v>0</v>
       </c>
       <c r="D4" s="4" t="n">
-        <f aca="false">COUNTIFS(Scenariusze!$B$2:$B$32,A4,Scenariusze!$H$2:$H$32,"Błąd")</f>
+        <f aca="false">COUNTIFS(Scenariusze!$B$2:$B$40,A4,Scenariusze!$H$2:$H$40,"Błąd")</f>
         <v>0</v>
       </c>
       <c r="E4" s="4" t="n">
         <f aca="false">B4-C4-D4</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F4" s="9" t="n">
         <f aca="false">IF(B4=0,0,(C4+D4)/B4)</f>
@@ -2349,18 +2673,18 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>149</v>
+        <v>169</v>
       </c>
       <c r="B5" s="4" t="n">
-        <f aca="false">COUNTIF(Scenariusze!$B$2:$B$32,A5)</f>
+        <f aca="false">COUNTIF(Scenariusze!$B$2:$B$40,A5)</f>
         <v>3</v>
       </c>
       <c r="C5" s="4" t="n">
-        <f aca="false">COUNTIFS(Scenariusze!$B$2:$B$32,A5,Scenariusze!$H$2:$H$32,"OK")</f>
+        <f aca="false">COUNTIFS(Scenariusze!$B$2:$B$40,A5,Scenariusze!$H$2:$H$40,"OK")</f>
         <v>0</v>
       </c>
       <c r="D5" s="4" t="n">
-        <f aca="false">COUNTIFS(Scenariusze!$B$2:$B$32,A5,Scenariusze!$H$2:$H$32,"Błąd")</f>
+        <f aca="false">COUNTIFS(Scenariusze!$B$2:$B$40,A5,Scenariusze!$H$2:$H$40,"Błąd")</f>
         <v>0</v>
       </c>
       <c r="E5" s="4" t="n">
@@ -2374,23 +2698,23 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>163</v>
+        <v>185</v>
       </c>
       <c r="B6" s="4" t="n">
-        <f aca="false">COUNTIF(Scenariusze!$B$2:$B$32,A6)</f>
-        <v>2</v>
+        <f aca="false">COUNTIF(Scenariusze!$B$2:$B$40,A6)</f>
+        <v>3</v>
       </c>
       <c r="C6" s="4" t="n">
-        <f aca="false">COUNTIFS(Scenariusze!$B$2:$B$32,A6,Scenariusze!$H$2:$H$32,"OK")</f>
+        <f aca="false">COUNTIFS(Scenariusze!$B$2:$B$40,A6,Scenariusze!$H$2:$H$40,"OK")</f>
         <v>0</v>
       </c>
       <c r="D6" s="4" t="n">
-        <f aca="false">COUNTIFS(Scenariusze!$B$2:$B$32,A6,Scenariusze!$H$2:$H$32,"Błąd")</f>
+        <f aca="false">COUNTIFS(Scenariusze!$B$2:$B$40,A6,Scenariusze!$H$2:$H$40,"Błąd")</f>
         <v>0</v>
       </c>
       <c r="E6" s="4" t="n">
         <f aca="false">B6-C6-D6</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F6" s="9" t="n">
         <f aca="false">IF(B6=0,0,(C6+D6)/B6)</f>
@@ -2398,40 +2722,65 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
-        <v>175</v>
-      </c>
-      <c r="B7" s="7" t="n">
-        <f aca="false">SUM(B2:B6)</f>
-        <v>31</v>
-      </c>
-      <c r="C7" s="7" t="n">
-        <f aca="false">SUM(C2:C6)</f>
+      <c r="A7" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="B7" s="4" t="n">
+        <f aca="false">COUNTIF(Scenariusze!$B$2:$B$40,A7)</f>
+        <v>2</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <f aca="false">COUNTIFS(Scenariusze!$B$2:$B$40,A7,Scenariusze!$H$2:$H$40,"OK")</f>
         <v>0</v>
       </c>
-      <c r="D7" s="7" t="n">
-        <f aca="false">SUM(D2:D6)</f>
+      <c r="D7" s="4" t="n">
+        <f aca="false">COUNTIFS(Scenariusze!$B$2:$B$40,A7,Scenariusze!$H$2:$H$40,"Błąd")</f>
         <v>0</v>
       </c>
-      <c r="E7" s="7" t="n">
-        <f aca="false">SUM(E2:E6)</f>
-        <v>31</v>
-      </c>
-      <c r="F7" s="10" t="n">
+      <c r="E7" s="4" t="n">
+        <f aca="false">B7-C7-D7</f>
+        <v>2</v>
+      </c>
+      <c r="F7" s="9" t="n">
         <f aca="false">IF(B7=0,0,(C7+D7)/B7)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
-        <v>176</v>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="B8" s="7" t="n">
+        <f aca="false">SUM(B2:B7)</f>
+        <v>39</v>
+      </c>
+      <c r="C8" s="7" t="n">
+        <f aca="false">SUM(C2:C7)</f>
+        <v>0</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <f aca="false">SUM(D2:D7)</f>
+        <v>0</v>
+      </c>
+      <c r="E8" s="7" t="n">
+        <f aca="false">SUM(E2:E7)</f>
+        <v>39</v>
+      </c>
+      <c r="F8" s="10" t="n">
+        <f aca="false">IF(B8=0,0,(C8+D8)/B8)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="E10" s="11" t="n">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="E11" s="11" t="n">
         <f aca="false">COUNTA(Błędy!$A$2:$A$500)-COUNTIF(Błędy!$L$2:$L$500,"sprawdzony")-COUNTIF(Błędy!$L$2:$L$500,"odrzucony")</f>
         <v>1</v>
       </c>
@@ -2478,79 +2827,79 @@
         <v>26</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>178</v>
+        <v>214</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>20</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>179</v>
+        <v>215</v>
       </c>
       <c r="F1" s="6" t="s">
         <v>21</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>180</v>
+        <v>216</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>181</v>
+        <v>217</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>182</v>
+        <v>218</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>183</v>
+        <v>219</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>184</v>
+        <v>220</v>
       </c>
       <c r="L1" s="6" t="s">
-        <v>185</v>
+        <v>221</v>
       </c>
       <c r="M1" s="6" t="s">
-        <v>186</v>
+        <v>222</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="12" t="s">
-        <v>187</v>
+        <v>223</v>
       </c>
       <c r="B2" s="13" t="n">
         <f aca="false">DATE(2026,10,16)</f>
         <v>46311</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>188</v>
+        <v>224</v>
       </c>
       <c r="D2" s="12" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>189</v>
+        <v>225</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="G2" s="12" t="s">
-        <v>190</v>
+        <v>226</v>
       </c>
       <c r="H2" s="12" t="s">
-        <v>191</v>
+        <v>227</v>
       </c>
       <c r="I2" s="12" t="s">
-        <v>192</v>
+        <v>228</v>
       </c>
       <c r="J2" s="12" t="s">
-        <v>193</v>
+        <v>229</v>
       </c>
       <c r="K2" s="12" t="s">
-        <v>194</v>
+        <v>230</v>
       </c>
       <c r="L2" s="12" t="s">
-        <v>195</v>
+        <v>231</v>
       </c>
       <c r="M2" s="12" t="s">
-        <v>196</v>
+        <v>232</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5571,73 +5920,73 @@
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>197</v>
+        <v>233</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>26</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>198</v>
+        <v>234</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>199</v>
+        <v>235</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>200</v>
+        <v>236</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>201</v>
+        <v>237</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>202</v>
+        <v>238</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>203</v>
+        <v>239</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>204</v>
+        <v>240</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>205</v>
+        <v>241</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="12" t="s">
-        <v>206</v>
+        <v>242</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>207</v>
+        <v>243</v>
       </c>
       <c r="C2" s="13" t="n">
         <f aca="false">DATE(2026,10,20)</f>
         <v>46315</v>
       </c>
       <c r="D2" s="12" t="s">
-        <v>208</v>
+        <v>244</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>209</v>
+        <v>245</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>210</v>
+        <v>246</v>
       </c>
       <c r="G2" s="12" t="s">
-        <v>211</v>
+        <v>247</v>
       </c>
       <c r="H2" s="12" t="s">
-        <v>212</v>
+        <v>248</v>
       </c>
       <c r="I2" s="12" t="s">
-        <v>213</v>
+        <v>249</v>
       </c>
       <c r="J2" s="12" t="s">
-        <v>214</v>
+        <v>250</v>
       </c>
       <c r="K2" s="12" t="s">
-        <v>215</v>
+        <v>251</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>